<commit_message>
fix(tests): updated constants in affected tests
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/10.1-solid-waste.xlsx
+++ b/packages/calculators/src/modules/test/10.1-solid-waste.xlsx
@@ -3,18 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B1E3CD2-329B-5E49-B469-EF2BDFED75AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2FDE9F-62D6-0D48-A01B-F475A1722B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15880" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="10.1" sheetId="4" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -318,6 +316,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="common"/>
+    </sheetNames>
+    <definedNames>
+      <definedName name="common_cch4" refersTo="='common'!$B$3"/>
+      <definedName name="common_cco2" refersTo="='common'!$B$2"/>
+    </definedNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="B2">
+            <v>3.67</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="B3">
+            <v>1.33</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -847,11 +873,11 @@
       </c>
       <c r="N5">
         <f t="shared" ref="N5:N10" si="5">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O5">
         <f>C5*M5*N5</f>
-        <v>555.5</v>
+        <v>556.005</v>
       </c>
       <c r="P5">
         <f t="shared" ref="P5:P10" si="6">$Y$9</f>
@@ -871,7 +897,7 @@
       </c>
       <c r="T5">
         <f>O5</f>
-        <v>555.5</v>
+        <v>556.005</v>
       </c>
       <c r="U5">
         <f>I5+S5</f>
@@ -894,8 +920,8 @@
         <v>20</v>
       </c>
       <c r="AC5">
-        <f>44/12</f>
-        <v>3.6666666666666665</v>
+        <f>[1]!common_cco2</f>
+        <v>3.67</v>
       </c>
       <c r="AE5" t="s">
         <v>6</v>
@@ -971,11 +997,11 @@
       </c>
       <c r="N6">
         <f t="shared" si="5"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O6">
         <f t="shared" ref="O6:O10" si="11">C6*M6*N6</f>
-        <v>185.16666666666666</v>
+        <v>185.33500000000001</v>
       </c>
       <c r="P6">
         <f t="shared" si="6"/>
@@ -995,7 +1021,7 @@
       </c>
       <c r="T6">
         <f t="shared" ref="T6:T10" si="13">O6</f>
-        <v>185.16666666666666</v>
+        <v>185.33500000000001</v>
       </c>
       <c r="U6">
         <f t="shared" ref="U6:U10" si="14">I6+S6</f>
@@ -1018,8 +1044,8 @@
         <v>62</v>
       </c>
       <c r="AC6">
-        <f>16/12</f>
-        <v>1.3333333333333333</v>
+        <f>[1]!common_cch4</f>
+        <v>1.33</v>
       </c>
       <c r="AE6" t="s">
         <v>4</v>
@@ -1086,11 +1112,11 @@
       </c>
       <c r="N7">
         <f t="shared" si="5"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O7">
         <f t="shared" si="11"/>
-        <v>228.49566666666669</v>
+        <v>228.70339000000001</v>
       </c>
       <c r="P7">
         <f t="shared" si="6"/>
@@ -1110,7 +1136,7 @@
       </c>
       <c r="T7">
         <f t="shared" si="13"/>
-        <v>228.49566666666669</v>
+        <v>228.70339000000001</v>
       </c>
       <c r="U7">
         <f t="shared" si="14"/>
@@ -1191,7 +1217,7 @@
       </c>
       <c r="N8">
         <f t="shared" si="5"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O8">
         <f t="shared" si="11"/>
@@ -1305,11 +1331,11 @@
       </c>
       <c r="N9">
         <f t="shared" si="5"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O9">
         <f t="shared" si="11"/>
-        <v>434.21583333333336</v>
+        <v>434.61057500000004</v>
       </c>
       <c r="P9">
         <f t="shared" si="6"/>
@@ -1329,7 +1355,7 @@
       </c>
       <c r="T9">
         <f t="shared" si="13"/>
-        <v>434.21583333333336</v>
+        <v>434.61057500000004</v>
       </c>
       <c r="U9">
         <f t="shared" si="14"/>
@@ -1422,7 +1448,7 @@
       </c>
       <c r="N10">
         <f t="shared" si="5"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="O10">
         <f t="shared" si="11"/>
@@ -1720,7 +1746,7 @@
       </c>
       <c r="O17">
         <f t="shared" ref="O17:O24" si="16">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P17">
         <f>IF(A17&lt;&gt;"Incineration", 0, F17*K17*L17*M17*N17*O17)</f>
@@ -1748,7 +1774,7 @@
       </c>
       <c r="V17">
         <f>$AC$6</f>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W17">
         <f>F17*Q17*R17*S17*T17*V17*(1-U17)</f>
@@ -1756,7 +1782,7 @@
       </c>
       <c r="X17">
         <f>SUM(P17:P26)</f>
-        <v>188.51871719999997</v>
+        <v>188.69009785199998</v>
       </c>
       <c r="Y17">
         <f>SUM(H17:H26,W17:W26)</f>
@@ -1819,11 +1845,11 @@
       </c>
       <c r="O18">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P18">
         <f t="shared" ref="P18:P24" si="24">IF(A18&lt;&gt;"Incineration", 0, F18*K18*L18*M18*N18*O18)</f>
-        <v>3.6860075999999999</v>
+        <v>3.689358516</v>
       </c>
       <c r="Q18">
         <f>_xlfn.XLOOKUP($B18,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -1847,7 +1873,7 @@
       </c>
       <c r="V18">
         <f t="shared" ref="V18:V56" si="26">$AC$6</f>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W18">
         <f t="shared" ref="W18:W24" si="27">F18*Q18*R18*S18*T18*V18*(1-U18)</f>
@@ -1906,7 +1932,7 @@
       </c>
       <c r="O19">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P19">
         <f t="shared" si="24"/>
@@ -1934,7 +1960,7 @@
       </c>
       <c r="V19">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W19">
         <f t="shared" si="27"/>
@@ -1993,7 +2019,7 @@
       </c>
       <c r="O20">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P20">
         <f t="shared" si="24"/>
@@ -2021,7 +2047,7 @@
       </c>
       <c r="V20">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W20">
         <f t="shared" si="27"/>
@@ -2080,7 +2106,7 @@
       </c>
       <c r="O21">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P21">
         <f t="shared" si="24"/>
@@ -2108,7 +2134,7 @@
       </c>
       <c r="V21">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W21">
         <f t="shared" si="27"/>
@@ -2167,11 +2193,11 @@
       </c>
       <c r="O22">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P22">
         <f t="shared" si="24"/>
-        <v>10.059280000000001</v>
+        <v>10.068424800000003</v>
       </c>
       <c r="Q22">
         <f>_xlfn.XLOOKUP($B22,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -2195,7 +2221,7 @@
       </c>
       <c r="V22">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W22">
         <f t="shared" si="27"/>
@@ -2254,7 +2280,7 @@
       </c>
       <c r="O23">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P23">
         <f t="shared" si="24"/>
@@ -2282,7 +2308,7 @@
       </c>
       <c r="V23">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W23">
         <f t="shared" si="27"/>
@@ -2341,11 +2367,11 @@
       </c>
       <c r="O24">
         <f t="shared" si="16"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P24">
         <f t="shared" si="24"/>
-        <v>9.2108015999999999</v>
+        <v>9.219175056000001</v>
       </c>
       <c r="Q24">
         <f>_xlfn.XLOOKUP($B24,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -2369,7 +2395,7 @@
       </c>
       <c r="V24">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W24">
         <f t="shared" si="27"/>
@@ -2428,11 +2454,11 @@
       </c>
       <c r="O25">
         <f t="shared" ref="O25:O26" si="33">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P25">
         <f>IF(A25&lt;&gt;"Incineration", 0, F25*K25*L25*M25*N25*O25)</f>
-        <v>165.56262799999996</v>
+        <v>165.71313947999997</v>
       </c>
       <c r="Q25">
         <f>_xlfn.XLOOKUP($B25,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -2456,7 +2482,7 @@
       </c>
       <c r="V25">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W25">
         <f t="shared" ref="W25:W26" si="34">F25*Q25*R25*S25*T25*V25*(1-U25)</f>
@@ -2516,7 +2542,7 @@
       </c>
       <c r="O26" s="3">
         <f t="shared" si="33"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P26" s="3">
         <f t="shared" ref="P26" si="35">IF(A26&lt;&gt;"Incineration", 0, F26*K26*L26*M26*N26*O26)</f>
@@ -2544,7 +2570,7 @@
       </c>
       <c r="V26" s="3">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W26" s="3">
         <f t="shared" si="34"/>
@@ -2606,7 +2632,7 @@
       </c>
       <c r="O27">
         <f t="shared" ref="O27:O34" si="36">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P27">
         <f>IF(A27&lt;&gt;"Incineration", 0, F27*K27*L27*M27*N27*O27)</f>
@@ -2634,11 +2660,11 @@
       </c>
       <c r="V27">
         <f>$AC$6</f>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W27">
         <f>F27*Q27*R27*S27*T27*V27*(1-U27)</f>
-        <v>82.924799999999991</v>
+        <v>82.717488000000003</v>
       </c>
       <c r="X27">
         <f>SUM(P27:P36)</f>
@@ -2646,7 +2672,7 @@
       </c>
       <c r="Y27">
         <f>SUM(H27:H36,W27:W36)</f>
-        <v>231.21257333333332</v>
+        <v>230.63454189999999</v>
       </c>
       <c r="Z27">
         <f>SUM(J27:J36)</f>
@@ -2705,7 +2731,7 @@
       </c>
       <c r="O28">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P28">
         <f t="shared" ref="P28:P36" si="42">IF(A28&lt;&gt;"Incineration", 0, F28*K28*L28*M28*N28*O28)</f>
@@ -2733,11 +2759,11 @@
       </c>
       <c r="V28">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W28">
         <f t="shared" ref="W28:W36" si="43">F28*Q28*R28*S28*T28*V28*(1-U28)</f>
-        <v>17.875200000000003</v>
+        <v>17.830512000000006</v>
       </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.2">
@@ -2792,7 +2818,7 @@
       </c>
       <c r="O29">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P29">
         <f t="shared" si="42"/>
@@ -2820,11 +2846,11 @@
       </c>
       <c r="V29">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W29">
         <f t="shared" si="43"/>
-        <v>13.660080000000001</v>
+        <v>13.6259298</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">
@@ -2879,7 +2905,7 @@
       </c>
       <c r="O30">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P30">
         <f t="shared" si="42"/>
@@ -2907,11 +2933,11 @@
       </c>
       <c r="V30">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W30">
         <f t="shared" si="43"/>
-        <v>32.909333333333336</v>
+        <v>32.827060000000003</v>
       </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.2">
@@ -2966,7 +2992,7 @@
       </c>
       <c r="O31">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P31">
         <f t="shared" si="42"/>
@@ -2994,11 +3020,11 @@
       </c>
       <c r="V31">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W31">
         <f t="shared" si="43"/>
-        <v>2.1242000000000001</v>
+        <v>2.1188895000000003</v>
       </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.2">
@@ -3053,7 +3079,7 @@
       </c>
       <c r="O32">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P32">
         <f t="shared" si="42"/>
@@ -3081,11 +3107,11 @@
       </c>
       <c r="V32">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W32">
         <f t="shared" si="43"/>
-        <v>2.4343199999999996</v>
+        <v>2.4282341999999999</v>
       </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.2">
@@ -3140,7 +3166,7 @@
       </c>
       <c r="O33">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P33">
         <f t="shared" si="42"/>
@@ -3168,11 +3194,11 @@
       </c>
       <c r="V33">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W33">
         <f t="shared" si="43"/>
-        <v>41.817599999999999</v>
+        <v>41.713056000000009</v>
       </c>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.2">
@@ -3227,7 +3253,7 @@
       </c>
       <c r="O34">
         <f t="shared" si="36"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P34">
         <f t="shared" si="42"/>
@@ -3255,11 +3281,11 @@
       </c>
       <c r="V34">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W34">
         <f t="shared" si="43"/>
-        <v>8.08704</v>
+        <v>8.0668224000000013</v>
       </c>
     </row>
     <row r="35" spans="1:26" x14ac:dyDescent="0.2">
@@ -3314,7 +3340,7 @@
       </c>
       <c r="O35">
         <f t="shared" ref="O35:O36" si="45">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P35">
         <f t="shared" si="42"/>
@@ -3342,11 +3368,11 @@
       </c>
       <c r="V35">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W35">
         <f t="shared" si="43"/>
-        <v>29.38</v>
+        <v>29.306550000000001</v>
       </c>
     </row>
     <row r="36" spans="1:26" x14ac:dyDescent="0.2">
@@ -3402,7 +3428,7 @@
       </c>
       <c r="O36" s="3">
         <f t="shared" si="45"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P36" s="3">
         <f t="shared" si="42"/>
@@ -3430,7 +3456,7 @@
       </c>
       <c r="V36" s="3">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W36" s="3">
         <f t="shared" si="43"/>
@@ -3492,7 +3518,7 @@
       </c>
       <c r="O37">
         <f t="shared" ref="O37:O44" si="46">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P37">
         <f>IF(A37&lt;&gt;"Incineration", 0, F37*K37*L37*M37*N37*O37)</f>
@@ -3520,7 +3546,7 @@
       </c>
       <c r="V37">
         <f>$AC$6</f>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W37">
         <f>F37*Q37*R37*S37*T37*V37*(1-U37)</f>
@@ -3528,11 +3554,11 @@
       </c>
       <c r="X37">
         <f>SUM(P37:P46)</f>
-        <v>547.28574999999978</v>
+        <v>547.78328249999993</v>
       </c>
       <c r="Y37">
         <f>SUM(H37:H46,W37:W46)</f>
-        <v>111.29263066666667</v>
+        <v>111.02520239</v>
       </c>
       <c r="Z37">
         <f>SUM(J37:J46)</f>
@@ -3591,7 +3617,7 @@
       </c>
       <c r="O38">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P38">
         <f t="shared" ref="P38:P46" si="52">IF(A38&lt;&gt;"Incineration", 0, F38*K38*L38*M38*N38*O38)</f>
@@ -3619,11 +3645,11 @@
       </c>
       <c r="V38">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W38">
         <f t="shared" ref="W38:W46" si="53">F38*Q38*R38*S38*T38*V38*(1-U38)</f>
-        <v>35.750400000000006</v>
+        <v>35.661024000000012</v>
       </c>
     </row>
     <row r="39" spans="1:26" x14ac:dyDescent="0.2">
@@ -3678,7 +3704,7 @@
       </c>
       <c r="O39">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P39">
         <f t="shared" si="52"/>
@@ -3706,7 +3732,7 @@
       </c>
       <c r="V39">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W39">
         <f t="shared" si="53"/>
@@ -3765,7 +3791,7 @@
       </c>
       <c r="O40">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P40">
         <f t="shared" si="52"/>
@@ -3793,11 +3819,11 @@
       </c>
       <c r="V40">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W40">
         <f t="shared" si="53"/>
-        <v>16.454666666666668</v>
+        <v>16.413530000000002</v>
       </c>
     </row>
     <row r="41" spans="1:26" x14ac:dyDescent="0.2">
@@ -3852,7 +3878,7 @@
       </c>
       <c r="O41">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P41">
         <f t="shared" si="52"/>
@@ -3880,11 +3906,11 @@
       </c>
       <c r="V41">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W41">
         <f t="shared" si="53"/>
-        <v>2.1242000000000001</v>
+        <v>2.1188895000000003</v>
       </c>
     </row>
     <row r="42" spans="1:26" x14ac:dyDescent="0.2">
@@ -3939,11 +3965,11 @@
       </c>
       <c r="O42">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P42">
         <f t="shared" si="52"/>
-        <v>10.059280000000001</v>
+        <v>10.068424800000003</v>
       </c>
       <c r="Q42">
         <f>_xlfn.XLOOKUP($B42,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -3967,7 +3993,7 @@
       </c>
       <c r="V42">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W42">
         <f t="shared" si="53"/>
@@ -4026,7 +4052,7 @@
       </c>
       <c r="O43">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P43">
         <f t="shared" si="52"/>
@@ -4054,7 +4080,7 @@
       </c>
       <c r="V43">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W43">
         <f t="shared" si="53"/>
@@ -4113,7 +4139,7 @@
       </c>
       <c r="O44">
         <f t="shared" si="46"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P44">
         <f t="shared" si="52"/>
@@ -4141,11 +4167,11 @@
       </c>
       <c r="V44">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W44">
         <f t="shared" si="53"/>
-        <v>6.3685439999999991</v>
+        <v>6.3526226399999999</v>
       </c>
     </row>
     <row r="45" spans="1:26" x14ac:dyDescent="0.2">
@@ -4200,7 +4226,7 @@
       </c>
       <c r="O45">
         <f t="shared" ref="O45:O46" si="55">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P45">
         <f t="shared" si="52"/>
@@ -4228,11 +4254,11 @@
       </c>
       <c r="V45">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W45">
         <f t="shared" si="53"/>
-        <v>46.273499999999991</v>
+        <v>46.157816249999996</v>
       </c>
     </row>
     <row r="46" spans="1:26" x14ac:dyDescent="0.2">
@@ -4288,11 +4314,11 @@
       </c>
       <c r="O46" s="3">
         <f t="shared" si="55"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P46" s="3">
         <f t="shared" si="52"/>
-        <v>537.22646999999984</v>
+        <v>537.71485769999992</v>
       </c>
       <c r="Q46" s="3">
         <f>_xlfn.XLOOKUP($B46,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -4316,7 +4342,7 @@
       </c>
       <c r="V46" s="3">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W46" s="3">
         <f t="shared" si="53"/>
@@ -4378,7 +4404,7 @@
       </c>
       <c r="O47">
         <f t="shared" ref="O47:O54" si="56">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P47">
         <f>IF(A47&lt;&gt;"Incineration", 0, F47*K47*L47*M47*N47*O47)</f>
@@ -4406,7 +4432,7 @@
       </c>
       <c r="V47">
         <f>$AC$6</f>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W47">
         <f>F47*Q47*R47*S47*T47*V47*(1-U47)</f>
@@ -4414,11 +4440,11 @@
       </c>
       <c r="X47">
         <f>SUM(P47:P56)</f>
-        <v>10.059280000000001</v>
+        <v>10.068424800000003</v>
       </c>
       <c r="Y47">
         <f>SUM(H47:H56,W47:W56)</f>
-        <v>90.003726666666665</v>
+        <v>89.790161900000015</v>
       </c>
       <c r="Z47">
         <f>SUM(J47:J56)</f>
@@ -4477,7 +4503,7 @@
       </c>
       <c r="O48">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P48">
         <f t="shared" ref="P48:P56" si="62">IF(A48&lt;&gt;"Incineration", 0, F48*K48*L48*M48*N48*O48)</f>
@@ -4505,7 +4531,7 @@
       </c>
       <c r="V48">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W48">
         <f t="shared" ref="W48:W56" si="63">F48*Q48*R48*S48*T48*V48*(1-U48)</f>
@@ -4564,7 +4590,7 @@
       </c>
       <c r="O49">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P49">
         <f t="shared" si="62"/>
@@ -4592,7 +4618,7 @@
       </c>
       <c r="V49">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W49">
         <f t="shared" si="63"/>
@@ -4651,7 +4677,7 @@
       </c>
       <c r="O50">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P50">
         <f t="shared" si="62"/>
@@ -4679,11 +4705,11 @@
       </c>
       <c r="V50">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W50">
         <f t="shared" si="63"/>
-        <v>16.454666666666668</v>
+        <v>16.413530000000002</v>
       </c>
     </row>
     <row r="51" spans="1:26" x14ac:dyDescent="0.2">
@@ -4738,7 +4764,7 @@
       </c>
       <c r="O51">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P51">
         <f t="shared" si="62"/>
@@ -4766,11 +4792,11 @@
       </c>
       <c r="V51">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W51">
         <f t="shared" si="63"/>
-        <v>2.1242000000000001</v>
+        <v>2.1188895000000003</v>
       </c>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.2">
@@ -4825,11 +4851,11 @@
       </c>
       <c r="O52">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P52">
         <f t="shared" si="62"/>
-        <v>10.059280000000001</v>
+        <v>10.068424800000003</v>
       </c>
       <c r="Q52">
         <f>_xlfn.XLOOKUP($B52,WasteEFs[w],WasteEFs[DOCw])</f>
@@ -4853,7 +4879,7 @@
       </c>
       <c r="V52">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W52">
         <f t="shared" si="63"/>
@@ -4912,7 +4938,7 @@
       </c>
       <c r="O53">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P53">
         <f t="shared" si="62"/>
@@ -4940,7 +4966,7 @@
       </c>
       <c r="V53">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W53">
         <f t="shared" si="63"/>
@@ -4999,7 +5025,7 @@
       </c>
       <c r="O54">
         <f t="shared" si="56"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P54">
         <f t="shared" si="62"/>
@@ -5027,11 +5053,11 @@
       </c>
       <c r="V54">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W54">
         <f t="shared" si="63"/>
-        <v>8.08704</v>
+        <v>8.0668224000000013</v>
       </c>
     </row>
     <row r="55" spans="1:26" x14ac:dyDescent="0.2">
@@ -5086,7 +5112,7 @@
       </c>
       <c r="O55">
         <f t="shared" ref="O55:O56" si="65">$AC$5</f>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P55">
         <f t="shared" si="62"/>
@@ -5114,11 +5140,11 @@
       </c>
       <c r="V55">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W55">
         <f t="shared" si="63"/>
-        <v>58.76</v>
+        <v>58.613100000000003</v>
       </c>
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.2">
@@ -5174,7 +5200,7 @@
       </c>
       <c r="O56" s="3">
         <f t="shared" si="65"/>
-        <v>3.6666666666666665</v>
+        <v>3.67</v>
       </c>
       <c r="P56" s="3">
         <f t="shared" si="62"/>
@@ -5202,7 +5228,7 @@
       </c>
       <c r="V56" s="3">
         <f t="shared" si="26"/>
-        <v>1.3333333333333333</v>
+        <v>1.33</v>
       </c>
       <c r="W56" s="3">
         <f t="shared" si="63"/>

</xml_diff>

<commit_message>
Update constants from NGAF (2024 to 2026) (#229)
* feat(scripts): basic NGAF extraction script + value updates

* fix(calculators): fixed double space in name and added stationary fuel values

* fix(calculators): updated incorrect anaerobic digestion constant

* fix(tests): updated constants in affected tests

* fix(calculators): updated references and JRPP value

* refactor(calculators): condensed constants from NGAF with functions

* chore: rebuilt schemas

* fix(scripts): added some comments re: PR feedback

* fix(calculators): split ngaf constants functions into separate file
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/10.1-solid-waste.xlsx
+++ b/packages/calculators/src/modules/test/10.1-solid-waste.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB77C36-C68E-D748-B59F-24285B8FDE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2FDE9F-62D6-0D48-A01B-F475A1722B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15880" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15880" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="10.1" sheetId="4" r:id="rId1"/>
@@ -849,11 +849,11 @@
       </c>
       <c r="H5">
         <f t="shared" ref="H5:H10" si="1">$Y$6</f>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I5">
         <f>A5*G5+B5*H5</f>
-        <v>0.95</v>
+        <v>2.75</v>
       </c>
       <c r="J5">
         <f t="shared" ref="J5:J10" si="2">$Z$5</f>
@@ -901,7 +901,7 @@
       </c>
       <c r="U5">
         <f>I5+S5</f>
-        <v>564.25</v>
+        <v>566.04999999999995</v>
       </c>
       <c r="V5">
         <f>L5</f>
@@ -973,11 +973,11 @@
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I6">
         <f t="shared" ref="I6:I10" si="9">A6*G6+B6*H6</f>
-        <v>0.85</v>
+        <v>1.75</v>
       </c>
       <c r="J6">
         <f t="shared" si="2"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="U6">
         <f t="shared" ref="U6:U10" si="14">I6+S6</f>
-        <v>115.65</v>
+        <v>116.55000000000001</v>
       </c>
       <c r="V6">
         <f t="shared" ref="V6:V10" si="15">L6</f>
@@ -1035,7 +1035,7 @@
         <v>9</v>
       </c>
       <c r="Y6">
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="Z6">
         <v>0</v>
@@ -1088,11 +1088,11 @@
       </c>
       <c r="H7">
         <f t="shared" si="1"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I7">
         <f t="shared" si="9"/>
-        <v>0.95</v>
+        <v>2.75</v>
       </c>
       <c r="J7">
         <f t="shared" si="2"/>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="U7">
         <f t="shared" si="14"/>
-        <v>0.95</v>
+        <v>2.75</v>
       </c>
       <c r="V7">
         <f t="shared" si="15"/>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I8">
         <f t="shared" si="9"/>
@@ -1307,11 +1307,11 @@
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I9">
         <f t="shared" si="9"/>
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="J9">
         <f t="shared" si="2"/>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="U9">
         <f t="shared" si="14"/>
-        <v>438</v>
+        <v>439.8</v>
       </c>
       <c r="V9">
         <f t="shared" si="15"/>
@@ -1424,11 +1424,11 @@
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="I10">
         <f t="shared" si="9"/>
-        <v>0.95</v>
+        <v>2.75</v>
       </c>
       <c r="J10">
         <f t="shared" si="2"/>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="U10">
         <f t="shared" si="14"/>
-        <v>564.25</v>
+        <v>566.04999999999995</v>
       </c>
       <c r="V10">
         <f t="shared" si="15"/>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="Y37">
         <f>SUM(H37:H46,W37:W46)</f>
-        <v>108.20251439</v>
+        <v>111.02520239</v>
       </c>
       <c r="Z37">
         <f>SUM(J37:J46)</f>
@@ -4020,11 +4020,11 @@
       </c>
       <c r="G43">
         <f t="shared" si="48"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="H43">
         <f t="shared" si="49"/>
-        <v>0.31363199999999997</v>
+        <v>3.1363199999999996</v>
       </c>
       <c r="I43">
         <f t="shared" si="50"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="Y47">
         <f>SUM(H47:H56,W47:W56)</f>
-        <v>86.967473900000016</v>
+        <v>89.790161900000015</v>
       </c>
       <c r="Z47">
         <f>SUM(J47:J56)</f>
@@ -4906,11 +4906,11 @@
       </c>
       <c r="G53">
         <f t="shared" si="58"/>
-        <v>1E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="H53">
         <f t="shared" si="59"/>
-        <v>0.31363199999999997</v>
+        <v>3.1363199999999996</v>
       </c>
       <c r="I53">
         <f t="shared" si="60"/>

</xml_diff>